<commit_message>
Add local work, ignore Result outputs
</commit_message>
<xml_diff>
--- a/Result/analyze_3.xlsx
+++ b/Result/analyze_3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,57 +436,47 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -497,36 +487,30 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -537,36 +521,30 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -577,36 +555,30 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -616,7 +588,9 @@
           <t>AI電力基建</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
@@ -639,12 +613,6 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -655,37 +623,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I6" t="n">
         <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -694,7 +656,9 @@
           <t>光學</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
@@ -711,18 +675,12 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -733,37 +691,31 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -773,37 +725,31 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>5</v>
-      </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I9" t="n">
         <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" t="n">
-        <v>7</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -812,35 +758,31 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
         <v>5</v>
       </c>
-      <c r="E10" t="n">
+      <c r="H10" t="n">
         <v>4</v>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" t="n">
-        <v>3</v>
-      </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" t="n">
-        <v>4</v>
-      </c>
-      <c r="L10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -851,37 +793,31 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" t="n">
         <v>5</v>
       </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" t="n">
-        <v>2</v>
-      </c>
       <c r="I11" t="n">
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -891,36 +827,30 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -934,34 +864,28 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -971,37 +895,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1011,37 +929,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="n">
-        <v>4</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -1051,36 +963,30 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H16" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" t="n">
-        <v>17</v>
-      </c>
-      <c r="L16" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1090,36 +996,32 @@
           <t>封裝測試</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>7</v>
+      </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
         <v>4</v>
       </c>
-      <c r="E17" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>4</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
       <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>8</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1128,15 +1030,17 @@
           <t>導線架</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1151,13 +1055,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1170,10 +1068,10 @@
         <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -1185,18 +1083,12 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1206,21 +1098,23 @@
           <t>工業自動化</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -1229,12 +1123,6 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1244,35 +1132,31 @@
           <t>工業電腦</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
         <v>4</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1282,12 +1166,14 @@
           <t>數位雲端</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -1299,18 +1185,12 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1330,13 +1210,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1345,13 +1225,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1360,12 +1234,14 @@
           <t>機器人</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1383,13 +1259,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1398,15 +1268,17 @@
           <t>橡膠</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1421,12 +1293,6 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1436,7 +1302,9 @@
           <t>水泥</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
       <c r="C26" t="n">
         <v>0</v>
       </c>
@@ -1459,12 +1327,6 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1474,12 +1336,14 @@
           <t>汽車</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
@@ -1488,7 +1352,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1498,12 +1362,6 @@
       </c>
       <c r="J27" t="n">
         <v>1</v>
-      </c>
-      <c r="K27" t="n">
-        <v>2</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1512,9 +1370,11 @@
           <t>油電燃氣</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -1526,21 +1386,15 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1551,10 +1405,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1569,19 +1423,13 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" t="n">
-        <v>2</v>
-      </c>
-      <c r="L29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1590,7 +1438,9 @@
           <t>玻璃</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
@@ -1613,12 +1463,6 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1628,35 +1472,31 @@
           <t>玻璃陶瓷</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1666,7 +1506,9 @@
           <t>生技</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
       <c r="C32" t="n">
         <v>0</v>
       </c>
@@ -1689,12 +1531,6 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1705,37 +1541,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" t="n">
         <v>4</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
-      </c>
-      <c r="K33" t="n">
-        <v>7</v>
-      </c>
-      <c r="L33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -1744,12 +1574,14 @@
           <t>石化</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -1764,16 +1596,10 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" t="n">
-        <v>1</v>
-      </c>
-      <c r="L34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1782,12 +1608,14 @@
           <t>紡織</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -1799,19 +1627,13 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
-      </c>
-      <c r="K35" t="n">
-        <v>4</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1820,36 +1642,32 @@
           <t>綠能</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
       <c r="C36" t="n">
         <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" t="n">
-        <v>1</v>
-      </c>
-      <c r="L36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -1858,36 +1676,32 @@
           <t>網通</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>2</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>2</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1896,7 +1710,9 @@
           <t>航空</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
@@ -1919,12 +1735,6 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1941,30 +1751,24 @@
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1975,37 +1779,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
       </c>
       <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="n">
+        <v>14</v>
+      </c>
+      <c r="J40" t="n">
         <v>4</v>
-      </c>
-      <c r="I40" t="n">
-        <v>1</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>2</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2021,10 +1819,10 @@
         <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -2040,12 +1838,6 @@
       </c>
       <c r="J41" t="n">
         <v>0</v>
-      </c>
-      <c r="K41" t="n">
-        <v>1</v>
-      </c>
-      <c r="L41" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -2054,12 +1846,14 @@
           <t>記憶體</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>3</v>
+      </c>
       <c r="C42" t="n">
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
@@ -2074,16 +1868,10 @@
         <v>2</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>6</v>
-      </c>
-      <c r="L42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -2093,37 +1881,31 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" t="n">
-        <v>1</v>
-      </c>
-      <c r="L43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2133,37 +1915,31 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2172,35 +1948,31 @@
           <t>軍工</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
       <c r="C45" t="n">
         <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2210,9 +1982,11 @@
           <t>農業科技</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -2233,12 +2007,6 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>1</v>
-      </c>
-      <c r="L46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2252,34 +2020,28 @@
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
         <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
-      </c>
-      <c r="K47" t="n">
-        <v>2</v>
-      </c>
-      <c r="L47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -2315,12 +2077,6 @@
       <c r="J48" t="n">
         <v>0</v>
       </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -2329,36 +2085,30 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
         <v>4</v>
       </c>
-      <c r="E49" t="n">
-        <v>5</v>
-      </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" t="n">
-        <v>2</v>
-      </c>
-      <c r="L49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2368,36 +2118,32 @@
           <t>運動休閒</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
-      </c>
-      <c r="K50" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="51">
@@ -2406,7 +2152,9 @@
           <t>醫療通路</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
       <c r="C51" t="n">
         <v>0</v>
       </c>
@@ -2429,12 +2177,6 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2448,10 +2190,10 @@
         <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
@@ -2463,18 +2205,12 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
-      </c>
-      <c r="K52" t="n">
-        <v>0</v>
-      </c>
-      <c r="L52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2485,37 +2221,31 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
         <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">
@@ -2524,7 +2254,9 @@
           <t>零售</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
       <c r="C54" t="n">
         <v>0</v>
       </c>
@@ -2547,12 +2279,6 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2562,7 +2288,9 @@
           <t>電信</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
+      <c r="B55" t="n">
+        <v>0</v>
+      </c>
       <c r="C55" t="n">
         <v>0</v>
       </c>
@@ -2585,12 +2313,6 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
-      </c>
-      <c r="K55" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2600,9 +2322,11 @@
           <t>電動車</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -2623,12 +2347,6 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2638,21 +2356,23 @@
           <t>電器電纜</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
+      <c r="B57" t="n">
+        <v>0</v>
+      </c>
       <c r="C57" t="n">
         <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -2661,12 +2381,6 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2676,12 +2390,14 @@
           <t>電子紙</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
       <c r="C58" t="n">
         <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
@@ -2699,12 +2415,6 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2714,15 +2424,17 @@
           <t>電子通路</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
+      <c r="B59" t="n">
+        <v>0</v>
+      </c>
       <c r="C59" t="n">
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -2731,18 +2443,12 @@
         <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
-      </c>
-      <c r="K59" t="n">
-        <v>3</v>
-      </c>
-      <c r="L59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2753,36 +2459,30 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C60" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D60" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I60" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
-      </c>
-      <c r="K60" t="n">
-        <v>4</v>
-      </c>
-      <c r="L60" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2796,34 +2496,28 @@
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
       </c>
       <c r="I61" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
-      </c>
-      <c r="K61" t="n">
-        <v>3</v>
-      </c>
-      <c r="L61" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2832,35 +2526,31 @@
           <t>電腦週邊</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
+      <c r="B62" t="n">
+        <v>5</v>
+      </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
-      </c>
-      <c r="K62" t="n">
-        <v>0</v>
-      </c>
-      <c r="L62" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2870,12 +2560,14 @@
           <t>面板</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
+      <c r="B63" t="n">
+        <v>0</v>
+      </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
@@ -2887,18 +2579,12 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" t="n">
-        <v>0</v>
-      </c>
-      <c r="L63" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2908,7 +2594,9 @@
           <t>食品</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
+      <c r="B64" t="n">
+        <v>0</v>
+      </c>
       <c r="C64" t="n">
         <v>0</v>
       </c>
@@ -2916,13 +2604,13 @@
         <v>0</v>
       </c>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2932,12 +2620,6 @@
       </c>
       <c r="J64" t="n">
         <v>0</v>
-      </c>
-      <c r="K64" t="n">
-        <v>0</v>
-      </c>
-      <c r="L64" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>